<commit_message>
Etappe 3: PDF-Import ohne KI – Modellauswahl, Fundstellen, Original-Vorschau, Synonyme
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwWy34XyZsiDiLNehTTTFj
</commit_message>
<xml_diff>
--- a/katalog/feldkatalog.xlsx
+++ b/katalog/feldkatalog.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Felder" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auswahlwerte" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wörterbuch" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Anleitung" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Felder" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Auswahlwerte" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Wörterbuch" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Synonyme" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Felder'!$A$1:$L$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Auswahlwerte'!$A$1:$E$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wörterbuch'!$A$1:$D$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Synonyme'!$A$1:$B$141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -560,63 +562,70 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>• Blatt „Synonyme“: wie ein Feld in Hersteller-Datenblättern heißen kann (hilft beim Auslesen ohne KI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>• Spalte „ID“ bitte NICHT ändern – darüber werden die Daten gespeichert.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Farben</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Hellblau = eines der 18 Kernfelder (müssen in Weclapp in jedem Fall stimmen, Pflichtprüfung in der Prüfmaske).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Hellblau = eines der 18 Kernfelder (müssen in Weclapp in jedem Fall stimmen, Pflichtprüfung in der Prüfmaske).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Gelb (Spalte Status) = Vorschlag von Claude, bitte prüfen und auf „bestätigt“ setzen.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Quellen (Spalte „Quelle“)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>F = Filter-Auswahl Produktkonfigurator · V = bisherige EPS-Vorlage (DE/EN) · P = EPS-Datenblattpaare 200034/200161/200326 · E = Pflichtenheft</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Beispiel</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Feld „Ausgangsspannung“: Datentyp „Bereich (von–bis)“, Einheit V. Im Datenblatt steht „0–750 V DC“; gespeichert wird zusätzlich min 0 / max 750 / V für den Filter.</t>
         </is>
@@ -7187,4 +7196,1715 @@
   <autoFilter ref="A1:D30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B141"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Feld-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Bezeichnung im Hersteller-Datenblatt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Ausgangsspannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Output voltage</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Output Voltage Range</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Nennspannung &amp; Bereich</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Nennspannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>DC Ausgang Spannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>DC-Ausgangsspannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Ausgangsspannungsbereich</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Gleichspannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Voltage output</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsspannung</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Rated output voltage</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsstrom</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Ausgangsstrom</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsstrom</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Output current</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsstrom</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Nennstrom &amp; Bereich</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsstrom</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Nennstrom</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsstrom</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>DC Ausgang Strom</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsstrom</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Rated output current</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsleistung</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Ausgangsleistung</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsleistung</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Output power</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsleistung</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Nennleistung &amp; Bereich</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsleistung</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Nennleistung</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsleistung</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Dauerausgangsleistung</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsleistung</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Rated power</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsleistung</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Continuous output power</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsleistung</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Output rating</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>eingangsspannung</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>AC Eingangsspannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>eingangsspannung</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>DC Eingangsspannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>eingangsspannung</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Eingangsspannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>eingangsspannung</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Input voltage</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>eingangsspannung</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Netzspannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>eingangsspannung</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Spannung / Phasen / Frequenz</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>eingangsspannung</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Mains voltage</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>eingangsspannung</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>AC input voltage</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>eingangsstrom</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Eingangsstrom</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>eingangsstrom</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Input current</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>eingangsfrequenz</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Eingangsfrequenz</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>eingangsfrequenz</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Input frequency</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>netzanschluss</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Netzanschluss</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>netzanschluss</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Mains</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>netzanschluss</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>AC-Anschluss</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>netzanschluss</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>AC input</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>leistungsfaktor</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Leistungsfaktor</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>leistungsfaktor</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Power factor</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>wirkungsgrad</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Wirkungsgrad</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>wirkungsgrad</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Efficiency</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>wirkungsgrad</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Effizienz</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>wirkungsgrad</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Effizienz max.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>betriebstemperatur</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Betriebstemperatur</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>betriebstemperatur</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Operating temperature</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>betriebstemperatur</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Operating temperature range</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>betriebstemperatur</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Operation temperature</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>betriebstemperatur</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Umgebungstemperatur</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>betriebstemperatur</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Arbeitstemperatur</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>lagertemperatur</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Lagertemperatur</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>lagertemperatur</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Storage temperature</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>luftfeuchtigkeit</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Luftfeuchtigkeit</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>luftfeuchtigkeit</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Humidity</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>luftfeuchtigkeit</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Relative humidity</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>luftfeuchtigkeit</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Rel. Luftfeuchte</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>betriebshoehe</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Betriebshöhe</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>betriebshoehe</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Altitude</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>betriebshoehe</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Aufstellhöhe</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>kuehlung</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Kühlung</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>kuehlung</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Cooling</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>kuehlung</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Kühlart</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>abmessungen</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Abmessungen</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>abmessungen</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Abmessungen (BxHxT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>abmessungen</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Abmessungen (B x H x T)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>abmessungen</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>abmessungen</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Package Dimensions (W x H x L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>abmessungen</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Dimensions (WxHxD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>abmessungen</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Maße</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>gewicht</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Gewicht</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>gewicht</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>gewicht</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Net weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>normen</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Normen</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>normen</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Standards</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>normen</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Sicherheitszertifikate</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>normen</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Zertifizierungen</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>schutzklasse</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Schutzklasse</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>schutzklasse</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Protection class</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>ueberspannungskategorie</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Überspannungskategorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>ueberspannungskategorie</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Overvoltage category</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>spannungsfestigkeit_ein_aus</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Isolation Eingang/Ausgang</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>spannungsfestigkeit_ein_aus</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Isolation In-/Output</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>spannungsfestigkeit_ein_aus</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Isolation input/output</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>anzeige</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Anzeige</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>anzeige</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>anzeige</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Anzeige und Bedieneinheit</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>betriebsarten</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Betriebsarten</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>betriebsarten</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Operation modes</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>betriebsarten</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Operating modes</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>betriebsarten</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Regelart</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>klirrfaktor</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Klirrfaktor</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>klirrfaktor</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>THD</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>klirrfaktor</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>Total Harmonic Distortion</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>scheitelfaktor</t>
+        </is>
+      </c>
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>Scheitelfaktor</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>scheitelfaktor</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>Crest factor</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>scheitelfaktor</t>
+        </is>
+      </c>
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Load Crest Factor</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsfrequenz</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Ausgangsfrequenz</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>ausgangsfrequenz</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Output frequency</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>restwelligkeit_i</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Restwelligkeit Strom</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>restwelligkeit_i</t>
+        </is>
+      </c>
+      <c r="B104" s="5" t="inlineStr">
+        <is>
+          <t>Ripple current</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>restwelligkeit_u</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Restwelligkeit Spannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>restwelligkeit_u</t>
+        </is>
+      </c>
+      <c r="B106" s="5" t="inlineStr">
+        <is>
+          <t>Restwelligkeit</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>restwelligkeit_u</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Restwelligkeit U</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>restwelligkeit_u</t>
+        </is>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
+          <t>Ripple</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>restwelligkeit_u</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Output Noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>spannungsstabilitaet_last</t>
+        </is>
+      </c>
+      <c r="B110" s="5" t="inlineStr">
+        <is>
+          <t>Spannungsstabilität Last</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>spannungsstabilitaet_last</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Load regulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>spannungsstabilitaet_last</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>Line/Load Regulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>spannungsstabilitaet_last</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Stabilität bei 0-100% Last</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
+        <is>
+          <t>spannungsstabilitaet_netz</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>Spannungsstabilität Netz</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>spannungsstabilitaet_netz</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Line regulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>spannungsstabilitaet_netz</t>
+        </is>
+      </c>
+      <c r="B116" s="5" t="inlineStr">
+        <is>
+          <t>Stabilität bei ±10% ∆ UAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>spannungsausregelung_last</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Spannungsausregelung Last</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
+        <is>
+          <t>spannungsausregelung_last</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
+          <t>Ausregelung 10-100% Last</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>spannungsausregelung_last</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>Transient response</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>anstiegszeit_spannung</t>
+        </is>
+      </c>
+      <c r="B120" s="5" t="inlineStr">
+        <is>
+          <t>Anstiegszeit Spannung</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>anstiegszeit_spannung</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>Anstiegszeit 10-90% UNenn</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>anstiegszeit_spannung</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="inlineStr">
+        <is>
+          <t>Rise time voltage</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>parallelschaltung</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Parallelschaltung</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>parallelschaltung</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>Parallel operation</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>parallelschaltung</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Parallelbetrieb</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>funktionsgenerator</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>Funktionsgenerator</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>funktionsgenerator</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>Function generator</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>netzrueckspeisung</t>
+        </is>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>Netzrückspeisung</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>netzrueckspeisung</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>Energy recovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>netzrueckspeisung</t>
+        </is>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>Energierückspeisung</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Artikelnummer</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>Part number</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Bestellnummer</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>Order code</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>Best.-Nr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>Art.-Nr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>Modell</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>MODEL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B141"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
0.3.1: Mausrad ändert keine Auswahlfelder mehr, „Model:“ wird gelesen, Gerätetyp-Vorschlag, weitere Synonyme
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwWy34XyZsiDiLNehTTTFj
</commit_message>
<xml_diff>
--- a/katalog/feldkatalog.xlsx
+++ b/katalog/feldkatalog.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Felder'!$A$1:$L$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Auswahlwerte'!$A$1:$E$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wörterbuch'!$A$1:$D$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Synonyme'!$A$1:$B$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Synonyme'!$A$1:$B$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7204,7 +7204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B141"/>
+  <dimension ref="A1:B147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8090,24 +8090,24 @@
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>gewicht</t>
+          <t>abmessungen</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>Gewicht</t>
+          <t>Package / Dimensions</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>gewicht</t>
+          <t>abmessungen</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>Weight</t>
+          <t>Package Dimensions</t>
         </is>
       </c>
     </row>
@@ -8119,31 +8119,31 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Net weight</t>
+          <t>Gewicht</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>normen</t>
+          <t>gewicht</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>Normen</t>
+          <t>Weight</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>normen</t>
+          <t>gewicht</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>Standards</t>
+          <t>Net weight</t>
         </is>
       </c>
     </row>
@@ -8155,7 +8155,7 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>Sicherheitszertifikate</t>
+          <t>Normen</t>
         </is>
       </c>
     </row>
@@ -8167,79 +8167,79 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Zertifizierungen</t>
+          <t>Standards</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>schutzklasse</t>
+          <t>normen</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>Schutzklasse</t>
+          <t>Sicherheitszertifikate</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>schutzklasse</t>
+          <t>normen</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>Protection class</t>
+          <t>Zertifizierungen</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>ueberspannungskategorie</t>
+          <t>schutzklasse</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>Überspannungskategorie</t>
+          <t>Schutzklasse</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>ueberspannungskategorie</t>
+          <t>schutzklasse</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>Overvoltage category</t>
+          <t>Protection class</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>spannungsfestigkeit_ein_aus</t>
+          <t>ueberspannungskategorie</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>Isolation Eingang/Ausgang</t>
+          <t>Überspannungskategorie</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>spannungsfestigkeit_ein_aus</t>
+          <t>ueberspannungskategorie</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>Isolation In-/Output</t>
+          <t>Overvoltage category</t>
         </is>
       </c>
     </row>
@@ -8251,31 +8251,31 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>Isolation input/output</t>
+          <t>Isolation Eingang/Ausgang</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>anzeige</t>
+          <t>spannungsfestigkeit_ein_aus</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Anzeige</t>
+          <t>Isolation In-/Output</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>anzeige</t>
+          <t>spannungsfestigkeit_ein_aus</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>Display</t>
+          <t>Isolation input/output</t>
         </is>
       </c>
     </row>
@@ -8287,223 +8287,223 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>Anzeige und Bedieneinheit</t>
+          <t>Anzeige</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>betriebsarten</t>
+          <t>anzeige</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>Betriebsarten</t>
+          <t>Display</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>betriebsarten</t>
+          <t>anzeige</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>Operation modes</t>
+          <t>Anzeige und Bedieneinheit</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>betriebsarten</t>
+          <t>anzeige</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>Operating modes</t>
+          <t>Indicators</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>betriebsarten</t>
+          <t>anzeige</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>Regelart</t>
+          <t>Anzeigen</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>klirrfaktor</t>
+          <t>betriebsarten</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>Klirrfaktor</t>
+          <t>Betriebsarten</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>klirrfaktor</t>
+          <t>betriebsarten</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>THD</t>
+          <t>Operation modes</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>klirrfaktor</t>
+          <t>betriebsarten</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>Total Harmonic Distortion</t>
+          <t>Operating modes</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>scheitelfaktor</t>
+          <t>betriebsarten</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>Scheitelfaktor</t>
+          <t>Regelart</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>scheitelfaktor</t>
+          <t>klirrfaktor</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>Crest factor</t>
+          <t>Klirrfaktor</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>scheitelfaktor</t>
+          <t>klirrfaktor</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>Load Crest Factor</t>
+          <t>THD</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>ausgangsfrequenz</t>
+          <t>klirrfaktor</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>Ausgangsfrequenz</t>
+          <t>Total Harmonic Distortion</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>ausgangsfrequenz</t>
+          <t>scheitelfaktor</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>Output frequency</t>
+          <t>Scheitelfaktor</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>restwelligkeit_i</t>
+          <t>scheitelfaktor</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>Restwelligkeit Strom</t>
+          <t>Crest factor</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>restwelligkeit_i</t>
+          <t>scheitelfaktor</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>Ripple current</t>
+          <t>Load Crest Factor</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>restwelligkeit_u</t>
+          <t>ausgangsfrequenz</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>Restwelligkeit Spannung</t>
+          <t>Ausgangsfrequenz</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>restwelligkeit_u</t>
+          <t>ausgangsfrequenz</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>Restwelligkeit</t>
+          <t>Output frequency</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>restwelligkeit_u</t>
+          <t>restwelligkeit_i</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>Restwelligkeit U</t>
+          <t>Restwelligkeit Strom</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>restwelligkeit_u</t>
+          <t>restwelligkeit_i</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Ripple current</t>
         </is>
       </c>
     </row>
@@ -8515,307 +8515,307 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>Output Noise</t>
+          <t>Restwelligkeit Spannung</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>spannungsstabilitaet_last</t>
+          <t>restwelligkeit_u</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>Spannungsstabilität Last</t>
+          <t>Restwelligkeit</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>spannungsstabilitaet_last</t>
+          <t>restwelligkeit_u</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>Load regulation</t>
+          <t>Restwelligkeit U</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>spannungsstabilitaet_last</t>
+          <t>restwelligkeit_u</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>Line/Load Regulation</t>
+          <t>Ripple</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>spannungsstabilitaet_last</t>
+          <t>restwelligkeit_u</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>Stabilität bei 0-100% Last</t>
+          <t>Output Noise</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>spannungsstabilitaet_netz</t>
+          <t>spannungsstabilitaet_last</t>
         </is>
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>Spannungsstabilität Netz</t>
+          <t>Spannungsstabilität Last</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>spannungsstabilitaet_netz</t>
+          <t>spannungsstabilitaet_last</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>Line regulation</t>
+          <t>Load regulation</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>spannungsstabilitaet_netz</t>
+          <t>spannungsstabilitaet_last</t>
         </is>
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>Stabilität bei ±10% ∆ UAC</t>
+          <t>Line/Load Regulation</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>spannungsausregelung_last</t>
+          <t>spannungsstabilitaet_last</t>
         </is>
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>Spannungsausregelung Last</t>
+          <t>Stabilität bei 0-100% Last</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>spannungsausregelung_last</t>
+          <t>spannungsstabilitaet_netz</t>
         </is>
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>Ausregelung 10-100% Last</t>
+          <t>Spannungsstabilität Netz</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>spannungsausregelung_last</t>
+          <t>spannungsstabilitaet_netz</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>Transient response</t>
+          <t>Line regulation</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>anstiegszeit_spannung</t>
+          <t>spannungsstabilitaet_netz</t>
         </is>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>Anstiegszeit Spannung</t>
+          <t>Stabilität bei ±10% ∆ UAC</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>anstiegszeit_spannung</t>
+          <t>spannungsausregelung_last</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>Anstiegszeit 10-90% UNenn</t>
+          <t>Spannungsausregelung Last</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>anstiegszeit_spannung</t>
+          <t>spannungsausregelung_last</t>
         </is>
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>Rise time voltage</t>
+          <t>Ausregelung 10-100% Last</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>parallelschaltung</t>
+          <t>spannungsausregelung_last</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
-          <t>Parallelschaltung</t>
+          <t>Transient response</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>parallelschaltung</t>
+          <t>anstiegszeit_spannung</t>
         </is>
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>Parallel operation</t>
+          <t>Anstiegszeit Spannung</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>parallelschaltung</t>
+          <t>anstiegszeit_spannung</t>
         </is>
       </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>Parallelbetrieb</t>
+          <t>Anstiegszeit 10-90% UNenn</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>funktionsgenerator</t>
+          <t>anstiegszeit_spannung</t>
         </is>
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>Funktionsgenerator</t>
+          <t>Rise time voltage</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>funktionsgenerator</t>
+          <t>parallelschaltung</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>Function generator</t>
+          <t>Parallelschaltung</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>netzrueckspeisung</t>
+          <t>parallelschaltung</t>
         </is>
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>Netzrückspeisung</t>
+          <t>Parallel operation</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>netzrueckspeisung</t>
+          <t>parallelschaltung</t>
         </is>
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>Energy recovery</t>
+          <t>Parallelbetrieb</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
         <is>
-          <t>netzrueckspeisung</t>
+          <t>funktionsgenerator</t>
         </is>
       </c>
       <c r="B130" s="5" t="inlineStr">
         <is>
-          <t>Energierückspeisung</t>
+          <t>Funktionsgenerator</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>hersteller_bestellnummer</t>
+          <t>funktionsgenerator</t>
         </is>
       </c>
       <c r="B131" s="5" t="inlineStr">
         <is>
-          <t>Artikelnummer</t>
+          <t>Function generator</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t>hersteller_bestellnummer</t>
+          <t>netzrueckspeisung</t>
         </is>
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>Part number</t>
+          <t>Netzrückspeisung</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>hersteller_bestellnummer</t>
+          <t>netzrueckspeisung</t>
         </is>
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>Bestellnummer</t>
+          <t>Energy recovery</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t>hersteller_bestellnummer</t>
+          <t>netzrueckspeisung</t>
         </is>
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>Order code</t>
+          <t>Energierückspeisung</t>
         </is>
       </c>
     </row>
@@ -8827,7 +8827,7 @@
       </c>
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>Best.-Nr.</t>
+          <t>Artikelnummer</t>
         </is>
       </c>
     </row>
@@ -8839,55 +8839,55 @@
       </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>Art.-Nr.</t>
+          <t>Part number</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>hersteller_typ</t>
+          <t>hersteller_bestellnummer</t>
         </is>
       </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Bestellnummer</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>hersteller_typ</t>
+          <t>hersteller_bestellnummer</t>
         </is>
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>Modell</t>
+          <t>Order code</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>hersteller_typ</t>
+          <t>hersteller_bestellnummer</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>Typ</t>
+          <t>Best.-Nr.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>hersteller_typ</t>
+          <t>hersteller_bestellnummer</t>
         </is>
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Art.-Nr.</t>
         </is>
       </c>
     </row>
@@ -8899,12 +8899,84 @@
       </c>
       <c r="B141" s="5" t="inlineStr">
         <is>
+          <t>Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>Modell</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
           <t>MODEL</t>
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>Model No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>Typenbezeichnung</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B141"/>
+  <autoFilter ref="A1:B147"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
v0.3.2: Ausgangsblock aufteilen (Strom/Leistung/Frequenz), Katalog-Synonyme nachladen, kompaktes PDF bei wenig Inhalt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwWy34XyZsiDiLNehTTTFj
</commit_message>
<xml_diff>
--- a/katalog/feldkatalog.xlsx
+++ b/katalog/feldkatalog.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Anleitung" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Felder" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Auswahlwerte" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Wörterbuch" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Synonyme" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Felder" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auswahlwerte" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wörterbuch" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synonyme" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Felder'!$A$1:$L$99</definedName>

</xml_diff>

<commit_message>
v0.3.3: Produktbilder aus dem PDF, Beschreibung/Produkttyp, abgeleitete Merkmale (Eingangsfrequenz, Bauform, Schutzfunktionen), Spaltengrenzen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwWy34XyZsiDiLNehTTTFj
</commit_message>
<xml_diff>
--- a/katalog/feldkatalog.xlsx
+++ b/katalog/feldkatalog.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anleitung" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Felder" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auswahlwerte" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wörterbuch" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synonyme" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Anleitung" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Felder" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Auswahlwerte" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Wörterbuch" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Synonyme" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Felder'!$A$1:$L$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Auswahlwerte'!$A$1:$E$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wörterbuch'!$A$1:$D$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Synonyme'!$A$1:$B$147</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Synonyme'!$A$1:$B$170</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7204,7 +7204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B147"/>
+  <dimension ref="A1:B170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8786,197 +8786,473 @@
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t>netzrueckspeisung</t>
+          <t>spannungsfestigkeit_aus_geh</t>
         </is>
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>Netzrückspeisung</t>
+          <t>Output to chassis</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>netzrueckspeisung</t>
+          <t>spannungsfestigkeit_aus_geh</t>
         </is>
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>Energy recovery</t>
+          <t>Output to case</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t>netzrueckspeisung</t>
+          <t>spannungsfestigkeit_aus_geh</t>
         </is>
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>Energierückspeisung</t>
+          <t>Ausgang zu Gehäuse</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>hersteller_bestellnummer</t>
+          <t>spannungsfestigkeit_aus_geh</t>
         </is>
       </c>
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>Artikelnummer</t>
+          <t>Ausgang/Gehäuse</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>hersteller_bestellnummer</t>
+          <t>robust</t>
         </is>
       </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>Part number</t>
+          <t>Ruggedizing</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>hersteller_bestellnummer</t>
+          <t>robust</t>
         </is>
       </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
-          <t>Bestellnummer</t>
+          <t>Ruggedized</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>hersteller_bestellnummer</t>
+          <t>robust</t>
         </is>
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>Order code</t>
+          <t>Robuste Ausführung</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>hersteller_bestellnummer</t>
+          <t>alarmmanagement</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>Best.-Nr.</t>
+          <t>Alarm Output</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>hersteller_bestellnummer</t>
+          <t>alarmmanagement</t>
         </is>
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>Art.-Nr.</t>
+          <t>Alarm output</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>hersteller_typ</t>
+          <t>alarmmanagement</t>
         </is>
       </c>
       <c r="B141" s="5" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Alarmausgang</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
         <is>
-          <t>hersteller_typ</t>
+          <t>alarmmanagement</t>
         </is>
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>Modell</t>
+          <t>Alarm</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="5" t="inlineStr">
         <is>
-          <t>hersteller_typ</t>
+          <t>begrenzung_ausgangsstrom</t>
         </is>
       </c>
       <c r="B143" s="5" t="inlineStr">
         <is>
-          <t>Typ</t>
+          <t>Output Overload Protection</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="5" t="inlineStr">
         <is>
-          <t>hersteller_typ</t>
+          <t>begrenzung_ausgangsstrom</t>
         </is>
       </c>
       <c r="B144" s="5" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Overload protection</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>hersteller_typ</t>
+          <t>begrenzung_ausgangsstrom</t>
         </is>
       </c>
       <c r="B145" s="5" t="inlineStr">
         <is>
-          <t>MODEL</t>
+          <t>Überlastschutz</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
         <is>
-          <t>hersteller_typ</t>
+          <t>einschaltstrombegrenzung</t>
         </is>
       </c>
       <c r="B146" s="5" t="inlineStr">
         <is>
-          <t>Model No.</t>
+          <t>Inrush current limiting</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="5" t="inlineStr">
         <is>
+          <t>einschaltstrombegrenzung</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>Inrush current limitation</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t>einschaltstrombegrenzung</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t>Einschaltstrombegrenzung</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>ueberhitzungsschutz</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>Over temperature protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="5" t="inlineStr">
+        <is>
+          <t>ueberhitzungsschutz</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="inlineStr">
+        <is>
+          <t>Overtemperature protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>ueberhitzungsschutz</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>Übertemperaturschutz</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>produkttyp</t>
+        </is>
+      </c>
+      <c r="B152" s="5" t="inlineStr">
+        <is>
+          <t>Summary description</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>beschreibung</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>Product description</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t>beschreibung</t>
+        </is>
+      </c>
+      <c r="B154" s="5" t="inlineStr">
+        <is>
+          <t>Produktbeschreibung</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>netzrueckspeisung</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>Netzrückspeisung</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>netzrueckspeisung</t>
+        </is>
+      </c>
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>Energy recovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>netzrueckspeisung</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>Energierückspeisung</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>Artikelnummer</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>Part number</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>Bestellnummer</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>Order code</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>Best.-Nr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_bestellnummer</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>Art.-Nr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
           <t>hersteller_typ</t>
         </is>
       </c>
-      <c r="B147" s="5" t="inlineStr">
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>Modell</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>MODEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>Model No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>hersteller_typ</t>
+        </is>
+      </c>
+      <c r="B170" s="5" t="inlineStr">
         <is>
           <t>Typenbezeichnung</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B147"/>
+  <autoFilter ref="A1:B170"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
v0.7.0: Formulierungs-Wörterbuch (Textbausteine in Werten, beide Richtungen), Werte vereinheitlichen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QwWy34XyZsiDiLNehTTTFj
</commit_message>
<xml_diff>
--- a/katalog/feldkatalog.xlsx
+++ b/katalog/feldkatalog.xlsx
@@ -11,13 +11,15 @@
     <sheet name="Felder" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Auswahlwerte" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Wörterbuch" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Synonyme" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Formulierungen" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Synonyme" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Felder'!$A$1:$L$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Auswahlwerte'!$A$1:$E$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Wörterbuch'!$A$1:$D$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Synonyme'!$A$1:$B$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Formulierungen'!$A$1:$C$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Synonyme'!$A$1:$B$170</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -555,77 +557,84 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>• Blatt „Wörterbuch“: Übersetzungen ergänzen oder korrigieren.</t>
+          <t>• Blatt „Wörterbuch“: Übersetzungen ganzer Werte ergänzen oder korrigieren.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>• Blatt „Synonyme“: wie ein Feld in Hersteller-Datenblättern heißen kann (hilft beim Auslesen ohne KI).</t>
+          <t>• Blatt „Formulierungen“: Textbausteine innerhalb eines Werts (z. B. „at full load“ = „bei Volllast“). Gilt in beide Richtungen.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>• Blatt „Synonyme“: wie ein Feld in Hersteller-Datenblättern heißen kann (hilft beim Auslesen ohne KI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>• Spalte „ID“ bitte NICHT ändern – darüber werden die Daten gespeichert.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Farben</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Hellblau = eines der 18 Kernfelder (müssen in Weclapp in jedem Fall stimmen, Pflichtprüfung in der Prüfmaske).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Hellblau = eines der 18 Kernfelder (müssen in Weclapp in jedem Fall stimmen, Pflichtprüfung in der Prüfmaske).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Gelb (Spalte Status) = Vorschlag von Claude, bitte prüfen und auf „bestätigt“ setzen.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Quellen (Spalte „Quelle“)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>F = Filter-Auswahl Produktkonfigurator · V = bisherige EPS-Vorlage (DE/EN) · P = EPS-Datenblattpaare 200034/200161/200326 · E = Pflichtenheft</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Beispiel</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Feld „Ausgangsspannung“: Datentyp „Bereich (von–bis)“, Einheit V. Im Datenblatt steht „0–750 V DC“; gespeichert wird zusätzlich min 0 / max 750 / V für den Filter.</t>
         </is>
@@ -7204,6 +7213,1038 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C76"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Englisch</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Bemerkung</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>from no load to full load</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>von Leerlauf bis Volllast</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>at full load</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>bei Volllast</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>10× in den Beispielen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>at 90% load</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>bei 90% Last</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>at no load</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>im Leerlauf</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>full load</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Volllast</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>no load</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Leerlauf</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>operating range</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Betriebsbereich</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>continuous</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>dauerhaft</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>z. B. 3000 W continuous</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>max per phase</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>max. pro Phase</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>per phase</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>pro Phase</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>for full specifications</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>bei voller Spezifikation</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>for full specification</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>bei voller Spezifikation</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>baseplate temperature</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Grundplattentemperatur</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>less than</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>kleiner als</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>better than</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>besser als</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>greater than</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>größer als</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>more than</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>mehr als</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>approximately</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>ca.</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>approx.</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>ca.</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>approx</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>ca.</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>maximum</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>maximal</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>minimum</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>typical</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>typisch</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>nominal</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>nominal</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>bleibt gleich (deutsch korrekt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>non-condensing</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>nicht kondensierend</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>non condensing</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>nicht kondensierend</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>current limiting with short circuit protection</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Strombegrenzung mit Kurzschlussschutz</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>thermal shutdown with automatic recovery</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>thermische Abschaltung mit automatischem Wiederanlauf</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>thermal shutdown</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>thermische Abschaltung</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>automatic recovery</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>automatischer Wiederanlauf</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>inrush current limiting</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Einschaltstrombegrenzung</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>current limiting</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Strombegrenzung</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>short circuit protection</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Kurzschlussschutz</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>short circuit proof</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>kurzschlussfest</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>overvoltage protection</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Überspannungsschutz</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>overtemperature protection</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Übertemperaturschutz</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>not installed</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>nicht vorhanden</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>air forced circulation with automatic fan speed regulation</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>forcierte Luftkühlung mit automatischer Lüfterdrehzahlregelung</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>air forced circulation</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>forcierte Luftkühlung</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>by built-in high quality internal fans</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>durch eingebaute hochwertige Lüfter</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>by built-in high quality fans</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>durch eingebaute hochwertige Lüfter</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>temperature controlled fans</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>temperaturgeregelte Lüfter</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>natural convection</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>natürliche Konvektion</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>water cooling</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Wasserkühlung</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>cooling slots</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Lüftungsschlitze</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>high frequency ripple is less than</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>HF-Restwelligkeit kleiner als</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>high frequency ripple is better than</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>HF-Restwelligkeit besser als</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Bandbreite</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>z. B. (20 MHz BW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>designed to meet</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>ausgelegt nach</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>and corresponding standards</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>und entsprechenden Normen</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>conformal coating</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Schutzlackierung</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>ruggedized</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>robuste Ausführung</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>ruggedizing</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>robuste Ausführung</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>chassis mount</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Chassismontage</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>rackmount</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Rack-Einbau</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>rack mount</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Rack-Einbau</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>output is floating</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Ausgang potentialfrei</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>floating</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>potentialfrei</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>galvanically isolated</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>galvanisch getrennt</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>adjustable</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>einstellbar</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>programmable</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>programmierbar</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>remote sensing</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Fernfühlung</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>output to chassis</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Ausgang zu Gehäuse</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>input to chassis</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>Eingang zu Gehäuse</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>input to output</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Eingang zu Ausgang</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>industrial quality sine wave inverter</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>Sinus-Wechselrichter in Industriequalität</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>industrial quality frequency converter</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Frequenzumformer in Industriequalität</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>sine wave inverter</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Sinus-Wechselrichter</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>frequency converter</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Frequenzumformer</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>DC/DC converter</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>DC/DC-Wandler</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>industrial quality</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Industriequalität</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>in case of insufficient cooling</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>bei unzureichender Kühlung</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>up to</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>bis zu</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>and</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>z. B. „UL 458 and EN 60950-1“</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C76"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>